<commit_message>
paper run 2026-08-30 06:28
</commit_message>
<xml_diff>
--- a/reports/2026-08-30.xlsx
+++ b/reports/2026-08-30.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,79 +628,111 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По активам</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -722,7 +754,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -744,7 +776,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -766,20 +798,64 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-08-30 17:49
</commit_message>
<xml_diff>
--- a/reports/2026-08-30.xlsx
+++ b/reports/2026-08-30.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -632,13 +632,13 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
         <v>1</v>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
       <c r="D15" t="n">
-        <v>-4.56</v>
+        <v>-4.65</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -654,17 +654,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
         <v>1</v>
       </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
       <c r="D17" t="n">
-        <v>-4.56</v>
+        <v>-0.09</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
@@ -673,40 +673,52 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-4.56</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>-4.56</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -716,45 +728,49 @@
         <v>0</v>
       </c>
       <c r="D21" t="n">
-        <v>-4.56</v>
+        <v>-4.34</v>
       </c>
       <c r="E21" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-4.65</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -776,7 +792,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -798,7 +814,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По цене входа</t>
+          <t>По часам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -820,7 +836,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По силе движения</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -842,20 +858,42 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>

</xml_diff>

<commit_message>
paper run 2026-08-30 23:46
</commit_message>
<xml_diff>
--- a/reports/2026-08-30.xlsx
+++ b/reports/2026-08-30.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,92 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-30T18:08:45.633477+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.61</v>
+      </c>
+      <c r="G2" t="n">
+        <v>9.029999999999999</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.00135</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>4.42</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-30T23:33:45.814440+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.797</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00239</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +593,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +603,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -536,6 +622,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +633,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +643,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="8">
@@ -573,6 +662,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +673,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>92.10000000000001</v>
+        <v>97.42000000000002</v>
       </c>
     </row>
     <row r="12">
@@ -647,174 +739,206 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5.32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-0.09</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
+          <t>По активам</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>-4.56</v>
+        <v>7.53</v>
       </c>
       <c r="E18" t="n">
-        <v>0</v>
+        <v>4.42</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" t="n">
         <v>2</v>
       </c>
-      <c r="C20" t="n">
-        <v>1</v>
-      </c>
       <c r="D20" t="n">
-        <v>-0.31</v>
+        <v>2.72</v>
       </c>
       <c r="E20" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" t="n">
-        <v>-4.34</v>
-      </c>
-      <c r="E21" t="n">
-        <v>0</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>5</v>
+      </c>
+      <c r="C22" t="n">
+        <v>4</v>
+      </c>
+      <c r="D22" t="n">
+        <v>11.88</v>
+      </c>
+      <c r="E22" t="n">
+        <v>5.32</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.55–0.60</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>3</v>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" t="n">
-        <v>-4.65</v>
+        <v>1.94</v>
       </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" t="n">
+        <v>2.18</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8.529999999999999</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5.32</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -831,72 +955,276 @@
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>BTC</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" t="n">
+        <v>4.42</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0.9</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" t="n">
+        <v>5.32</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>4.42</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2</v>
+      </c>
+      <c r="C43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" t="n">
+        <v>5.32</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>4.42</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0.20%+</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>4.42</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>